<commit_message>
feat: added vertex and triangle tracker
Added VertexCounter script which calculates the amount of vertices and triangles in the scene.

Updated the report document with an explanation of tessellation factor.
Updated the Data file with the amount of vertices and triangle from the first tests
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Year 2\TesselationTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E319B85E-D70A-41F1-BFFD-BDBEEB22E5C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8052E586-CB76-4724-8844-F2333159CD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Test 1</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Average (FPS)</t>
   </si>
   <si>
-    <t>No tessellation</t>
-  </si>
-  <si>
     <t>Tessellation factor 4</t>
   </si>
   <si>
@@ -102,6 +99,15 @@
   </si>
   <si>
     <t>10x10 City; Seed 2; Min 3 Height; Max 5 Height</t>
+  </si>
+  <si>
+    <t>Tessellation factor 1 (no tesselation)</t>
+  </si>
+  <si>
+    <t>Triangle Count</t>
+  </si>
+  <si>
+    <t>Vertex Count</t>
   </si>
 </sst>
 </file>
@@ -143,9 +149,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,16 +433,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="1" max="1" width="39.44140625" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -449,10 +458,16 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>99.74</v>
@@ -467,10 +482,16 @@
         <f>AVERAGE(B2:D2)</f>
         <v>99.236666666666665</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H2" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>95.07</v>
@@ -485,10 +506,16 @@
         <f t="shared" ref="E3:E18" si="0">AVERAGE(B3:D3)</f>
         <v>94.11</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G3" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H3" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>94.57</v>
@@ -503,10 +530,16 @@
         <f t="shared" si="0"/>
         <v>93.686666666666667</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H4" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>90.85</v>
@@ -521,10 +554,16 @@
         <f t="shared" si="0"/>
         <v>90.95</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G5" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H5" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>91.52</v>
@@ -539,113 +578,191 @@
         <f t="shared" si="0"/>
         <v>90.726666666666674</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G6" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H6" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G7" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H7" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="E8" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G8" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H8" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="E9" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H9" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="E10" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G10" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H10" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="E11" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G11" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H11" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="E12" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G12" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H12" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="E13" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G13" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H13" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="E14" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G14" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H14" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="E15" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G15" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H15" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="E16" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G16" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H16" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="E16" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="E17" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="G17" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H17" s="2">
+        <v>8321936</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>20</v>
-      </c>
       <c r="E18" s="1" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
+      </c>
+      <c r="G18" s="2">
+        <v>5183814</v>
+      </c>
+      <c r="H18" s="2">
+        <v>8321936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: track data for tessellation factor 20 to 64
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,13 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Year 2\TesselationTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8052E586-CB76-4724-8844-F2333159CD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CFD78D-3801-49D5-B665-578D9141E506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$A$2:$A$18</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$E$2:$E$18</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$J$2</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$M$6</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$M$6</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Test 1</t>
   </si>
@@ -47,67 +54,19 @@
     <t>Test 3</t>
   </si>
   <si>
-    <t>Average (FPS)</t>
-  </si>
-  <si>
-    <t>Tessellation factor 4</t>
-  </si>
-  <si>
-    <t>Tessellation factor 8</t>
-  </si>
-  <si>
-    <t>Tessellation factor 12</t>
-  </si>
-  <si>
-    <t>Tessellation factor 16</t>
-  </si>
-  <si>
-    <t>Tessellation factor 20</t>
-  </si>
-  <si>
-    <t>Tessellation factor 24</t>
-  </si>
-  <si>
-    <t>Tessellationfactor 28</t>
-  </si>
-  <si>
-    <t>Tessellation factor 32</t>
-  </si>
-  <si>
-    <t>Tessellation factor 36</t>
-  </si>
-  <si>
-    <t>Tessellation factor 40</t>
-  </si>
-  <si>
-    <t>Tessellation factor 44</t>
-  </si>
-  <si>
-    <t>Tessellation factor 48</t>
-  </si>
-  <si>
-    <t>Tessellation factor 52</t>
-  </si>
-  <si>
-    <t>Tessellation factor 56</t>
-  </si>
-  <si>
-    <t>Tessellation factor 60</t>
-  </si>
-  <si>
-    <t>Tessellationfactor 64</t>
-  </si>
-  <si>
     <t>10x10 City; Seed 2; Min 3 Height; Max 5 Height</t>
-  </si>
-  <si>
-    <t>Tessellation factor 1 (no tesselation)</t>
   </si>
   <si>
     <t>Triangle Count</t>
   </si>
   <si>
     <t>Vertex Count</t>
+  </si>
+  <si>
+    <t>Tessellation factor</t>
+  </si>
+  <si>
+    <t>Average FPS</t>
   </si>
 </sst>
 </file>
@@ -149,10 +108,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -168,6 +128,1117 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>FPS across tessellatio</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t>n factors</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.2597845581802275"/>
+          <c:y val="0"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>FPS</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$18</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>56</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>64</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$2:$E$18</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="17"/>
+                <c:pt idx="0">
+                  <c:v>99.236666666666665</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>94.11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>93.686666666666667</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>90.95</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>90.726666666666674</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>90.613333333333344</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>89.17</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>87.12</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>85.490000000000009</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>83.306666666666672</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>81.583333333333329</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>80.25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>78.486666666666665</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>76.516666666666666</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>74.796666666666667</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>73.073333333333323</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>71.463333333333338</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-77AC-4262-BA97-365C23CC0218}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="316393616"/>
+        <c:axId val="316395056"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="316393616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Tessellation factor</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="316395056"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="316395056"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Average FPS</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="316393616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87DCC73D-A7D5-4D22-1163-AD721A04576F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -433,18 +1504,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.44140625" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
     <col min="7" max="7" width="15.88671875" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -456,18 +1527,21 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" t="s">
-        <v>23</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>21</v>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
       </c>
       <c r="B2">
         <v>99.74</v>
@@ -489,8 +1563,8 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
         <v>4</v>
       </c>
       <c r="B3">
@@ -513,9 +1587,9 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>8</v>
       </c>
       <c r="B4">
         <v>94.57</v>
@@ -537,9 +1611,9 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>6</v>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>12</v>
       </c>
       <c r="B5">
         <v>90.85</v>
@@ -561,9 +1635,9 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>7</v>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>16</v>
       </c>
       <c r="B6">
         <v>91.52</v>
@@ -585,13 +1659,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="1" t="e">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>90.97</v>
+      </c>
+      <c r="C7">
+        <v>89.93</v>
+      </c>
+      <c r="D7">
+        <v>90.94</v>
+      </c>
+      <c r="E7" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>90.613333333333344</v>
       </c>
       <c r="G7" s="2">
         <v>5183814</v>
@@ -600,13 +1683,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="1" t="e">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>24</v>
+      </c>
+      <c r="B8">
+        <v>89.56</v>
+      </c>
+      <c r="C8">
+        <v>89.16</v>
+      </c>
+      <c r="D8">
+        <v>88.79</v>
+      </c>
+      <c r="E8" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>89.17</v>
       </c>
       <c r="G8" s="2">
         <v>5183814</v>
@@ -615,13 +1707,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="1" t="e">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>28</v>
+      </c>
+      <c r="B9">
+        <v>87.2</v>
+      </c>
+      <c r="C9">
+        <v>87.08</v>
+      </c>
+      <c r="D9">
+        <v>87.08</v>
+      </c>
+      <c r="E9" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>87.12</v>
       </c>
       <c r="G9" s="2">
         <v>5183814</v>
@@ -630,13 +1731,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="1" t="e">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>32</v>
+      </c>
+      <c r="B10">
+        <v>85.65</v>
+      </c>
+      <c r="C10">
+        <v>85.33</v>
+      </c>
+      <c r="D10">
+        <v>85.49</v>
+      </c>
+      <c r="E10" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>85.490000000000009</v>
       </c>
       <c r="G10" s="2">
         <v>5183814</v>
@@ -645,13 +1755,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" s="1" t="e">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>36</v>
+      </c>
+      <c r="B11">
+        <v>83.69</v>
+      </c>
+      <c r="C11">
+        <v>83.34</v>
+      </c>
+      <c r="D11">
+        <v>82.89</v>
+      </c>
+      <c r="E11" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>83.306666666666672</v>
       </c>
       <c r="G11" s="2">
         <v>5183814</v>
@@ -660,13 +1779,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="E12" s="1" t="e">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>40</v>
+      </c>
+      <c r="B12">
+        <v>81.59</v>
+      </c>
+      <c r="C12">
+        <v>81.459999999999994</v>
+      </c>
+      <c r="D12">
+        <v>81.7</v>
+      </c>
+      <c r="E12" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>81.583333333333329</v>
       </c>
       <c r="G12" s="2">
         <v>5183814</v>
@@ -675,13 +1803,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="1" t="e">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>44</v>
+      </c>
+      <c r="B13">
+        <v>80.37</v>
+      </c>
+      <c r="C13">
+        <v>80.25</v>
+      </c>
+      <c r="D13">
+        <v>80.13</v>
+      </c>
+      <c r="E13" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>80.25</v>
       </c>
       <c r="G13" s="2">
         <v>5183814</v>
@@ -690,13 +1827,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="1" t="e">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>48</v>
+      </c>
+      <c r="B14">
+        <v>78.849999999999994</v>
+      </c>
+      <c r="C14">
+        <v>78.430000000000007</v>
+      </c>
+      <c r="D14">
+        <v>78.180000000000007</v>
+      </c>
+      <c r="E14" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>78.486666666666665</v>
       </c>
       <c r="G14" s="2">
         <v>5183814</v>
@@ -705,13 +1851,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="1" t="e">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>52</v>
+      </c>
+      <c r="B15">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="C15">
+        <v>76.5</v>
+      </c>
+      <c r="D15">
+        <v>76.45</v>
+      </c>
+      <c r="E15" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>76.516666666666666</v>
       </c>
       <c r="G15" s="2">
         <v>5183814</v>
@@ -720,13 +1875,22 @@
         <v>8321936</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="1" t="e">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>56</v>
+      </c>
+      <c r="B16">
+        <v>74.930000000000007</v>
+      </c>
+      <c r="C16">
+        <v>74.760000000000005</v>
+      </c>
+      <c r="D16">
+        <v>74.7</v>
+      </c>
+      <c r="E16" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>74.796666666666667</v>
       </c>
       <c r="G16" s="2">
         <v>5183814</v>
@@ -736,12 +1900,21 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="1" t="e">
+      <c r="A17" s="3">
+        <v>60</v>
+      </c>
+      <c r="B17">
+        <v>73.239999999999995</v>
+      </c>
+      <c r="C17">
+        <v>73.02</v>
+      </c>
+      <c r="D17">
+        <v>72.959999999999994</v>
+      </c>
+      <c r="E17" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>73.073333333333323</v>
       </c>
       <c r="G17" s="2">
         <v>5183814</v>
@@ -751,12 +1924,21 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="1" t="e">
+      <c r="A18" s="3">
+        <v>64</v>
+      </c>
+      <c r="B18">
+        <v>71.53</v>
+      </c>
+      <c r="C18">
+        <v>71.45</v>
+      </c>
+      <c r="D18">
+        <v>71.41</v>
+      </c>
+      <c r="E18" s="1">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>71.463333333333338</v>
       </c>
       <c r="G18" s="2">
         <v>5183814</v>
@@ -768,5 +1950,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: track data for chart 2
Tracked framerate across different city sizes.
From 3x3 to 18x18.

chore: took images for each city size
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,20 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Year 2\TesselationTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0CFD78D-3801-49D5-B665-578D9141E506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCEB62A6-0272-48EF-B6CD-20565997B099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tessellation Factors" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$A$2:$A$18</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$E$2:$E$18</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$J$2</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$M$6</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$M$6</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
   <si>
     <t>Test 1</t>
   </si>
@@ -68,11 +62,44 @@
   <si>
     <t>Average FPS</t>
   </si>
+  <si>
+    <t>Triangle Count (in millions)</t>
+  </si>
+  <si>
+    <t>Rows and Columns</t>
+  </si>
+  <si>
+    <t>15x15</t>
+  </si>
+  <si>
+    <t>3x3</t>
+  </si>
+  <si>
+    <t>6x6</t>
+  </si>
+  <si>
+    <t>9x9</t>
+  </si>
+  <si>
+    <t>12x12</t>
+  </si>
+  <si>
+    <t>18x18</t>
+  </si>
+  <si>
+    <t>21x21</t>
+  </si>
+  <si>
+    <t>crashes</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.000,,"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -108,11 +135,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -238,7 +266,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$18</c:f>
+              <c:f>'Tessellation Factors'!$A$2:$A$18</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="17"/>
@@ -298,7 +326,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$18</c:f>
+              <c:f>'Tessellation Factors'!$E$2:$E$18</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="17"/>
@@ -644,7 +672,490 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>FPS across city sizes</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Average FPS</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.000,,</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>446196</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2557912</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6588388</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12503168</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20099300</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>29901464</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$F$2:$F$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>115.24666666666667</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>106.07333333333334</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>96.173333333333332</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>80.926666666666677</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>68.02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>56.973333333333329</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-25C9-4CE3-89B2-C5FC0CC3035C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1988097360"/>
+        <c:axId val="1988095440"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1988097360"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Triangles in scene (in millions)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0.000,," sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1988095440"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1988095440"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Average</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>FPS</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1988097360"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1200,6 +1711,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1221,6 +2248,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{87DCC73D-A7D5-4D22-1163-AD721A04576F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>312420</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BF8B72D-AB5A-5E10-0B84-0CCDBEF3D45F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1507,7 +2575,7 @@
   <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.109375" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
     <col min="7" max="7" width="15.88671875" customWidth="1"/>
     <col min="8" max="8" width="13" customWidth="1"/>
@@ -1530,10 +2598,10 @@
         <v>7</v>
       </c>
       <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
         <v>4</v>
-      </c>
-      <c r="H1" t="s">
-        <v>5</v>
       </c>
       <c r="J1" t="s">
         <v>3</v>
@@ -1952,4 +3020,212 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0519DB-39C6-4963-B577-A1DDE442233F}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.5546875" customWidth="1"/>
+    <col min="2" max="2" width="26.21875" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="17.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="4">
+        <v>446196</v>
+      </c>
+      <c r="C2">
+        <v>115.9</v>
+      </c>
+      <c r="D2">
+        <v>115.21</v>
+      </c>
+      <c r="E2">
+        <v>114.63</v>
+      </c>
+      <c r="F2" s="1">
+        <f>AVERAGE(C2:E2)</f>
+        <v>115.24666666666667</v>
+      </c>
+      <c r="H2" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4">
+        <v>2557912</v>
+      </c>
+      <c r="C3">
+        <v>106.71</v>
+      </c>
+      <c r="D3">
+        <v>106.04</v>
+      </c>
+      <c r="E3">
+        <v>105.47</v>
+      </c>
+      <c r="F3" s="1">
+        <f t="shared" ref="F3:F8" si="0">AVERAGE(C3:E3)</f>
+        <v>106.07333333333334</v>
+      </c>
+      <c r="H3" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4">
+        <v>6588388</v>
+      </c>
+      <c r="C4">
+        <v>96.89</v>
+      </c>
+      <c r="D4">
+        <v>96.23</v>
+      </c>
+      <c r="E4">
+        <v>95.4</v>
+      </c>
+      <c r="F4" s="1">
+        <f t="shared" si="0"/>
+        <v>96.173333333333332</v>
+      </c>
+      <c r="H4" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="4">
+        <v>12503168</v>
+      </c>
+      <c r="C5">
+        <v>80.97</v>
+      </c>
+      <c r="D5">
+        <v>81.260000000000005</v>
+      </c>
+      <c r="E5">
+        <v>80.55</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" si="0"/>
+        <v>80.926666666666677</v>
+      </c>
+      <c r="H5" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4">
+        <v>20099300</v>
+      </c>
+      <c r="C6">
+        <v>67.88</v>
+      </c>
+      <c r="D6">
+        <v>68.77</v>
+      </c>
+      <c r="E6">
+        <v>67.41</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="0"/>
+        <v>68.02</v>
+      </c>
+      <c r="H6" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4">
+        <v>29901464</v>
+      </c>
+      <c r="C7">
+        <v>58.03</v>
+      </c>
+      <c r="D7">
+        <v>56.73</v>
+      </c>
+      <c r="E7">
+        <v>56.16</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="0"/>
+        <v>56.973333333333329</v>
+      </c>
+      <c r="H7" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4">
+        <v>40374324</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="3">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: added a collage of all the tessellation factor images and city images
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Year 2\TesselationTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCEB62A6-0272-48EF-B6CD-20565997B099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11F2A50-DB99-46AB-B7C6-B6E962345F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tessellation Factors" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Cities" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -767,7 +767,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet2!$B$2:$B$7</c:f>
+              <c:f>Cities!$B$2:$B$7</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.000,,</c:formatCode>
                 <c:ptCount val="6"/>
@@ -794,7 +794,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$F$2:$F$7</c:f>
+              <c:f>Cities!$F$2:$F$7</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -3098,7 +3098,7 @@
         <v>105.47</v>
       </c>
       <c r="F3" s="1">
-        <f t="shared" ref="F3:F8" si="0">AVERAGE(C3:E3)</f>
+        <f t="shared" ref="F3:F7" si="0">AVERAGE(C3:E3)</f>
         <v>106.07333333333334</v>
       </c>
       <c r="H3" s="3">

</xml_diff>

<commit_message>
fix: switched to correct picture for chart2
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Year 2\TesselationTesting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B11F2A50-DB99-46AB-B7C6-B6E962345F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46541822-6F17-48C1-B8B2-74F02B14B451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>Test 1</t>
   </si>
@@ -87,10 +87,7 @@
     <t>18x18</t>
   </si>
   <si>
-    <t>21x21</t>
-  </si>
-  <si>
-    <t>crashes</t>
+    <t>No tessellation</t>
   </si>
 </sst>
 </file>
@@ -706,7 +703,14 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
               <a:t>FPS across city sizes</a:t>
             </a:r>
           </a:p>
@@ -744,30 +748,135 @@
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Average FPS</c:v>
+            <c:v>TF1</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
+          <c:invertIfNegative val="0"/>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="25400" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:cat>
             <c:numRef>
-              <c:f>Cities!$B$2:$B$7</c:f>
+              <c:f>Cities!$B$11:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0.000,,</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>446196</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2557912</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6588388</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12503168</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20099300</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>29901464</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Cities!$F$11:$F$16</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>119.69</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>109.31666666666666</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>91.446666666666673</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>79.733333333333334</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>73.056666666666672</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>65.95</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FDA7-46A1-B02D-CDB22048C60C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>TF20</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="25400" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:cat>
+            <c:numRef>
+              <c:f>Cities!$B$11:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.000,,</c:formatCode>
                 <c:ptCount val="6"/>
@@ -799,30 +908,29 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>115.24666666666667</c:v>
+                  <c:v>118.44333333333333</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>106.07333333333334</c:v>
+                  <c:v>104.99333333333334</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>96.173333333333332</c:v>
+                  <c:v>88.256666666666661</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>80.926666666666677</c:v>
+                  <c:v>76.59</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>68.02</c:v>
+                  <c:v>71.163333333333341</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>56.973333333333329</c:v>
+                  <c:v>65.073333333333338</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-25C9-4CE3-89B2-C5FC0CC3035C}"/>
+              <c16:uniqueId val="{00000002-FDA7-46A1-B02D-CDB22048C60C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -834,12 +942,13 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="1988097360"/>
-        <c:axId val="1988095440"/>
-      </c:lineChart>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1465790543"/>
+        <c:axId val="1465784783"/>
+      </c:barChart>
       <c:catAx>
-        <c:axId val="1988097360"/>
+        <c:axId val="1465790543"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -866,8 +975,13 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>Triangles in scene (in millions)</a:t>
+                  <a:t>Triangles</a:t>
                 </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> in scene (in millions)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -937,7 +1051,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1988095440"/>
+        <c:crossAx val="1465784783"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -945,7 +1059,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1988095440"/>
+        <c:axId val="1465784783"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -986,15 +1100,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>Average</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" baseline="0"/>
-                  <a:t> </a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>FPS</a:t>
+                  <a:t>Average FPS</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1059,7 +1165,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1988097360"/>
+        <c:crossAx val="1465790543"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1071,6 +1177,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -1712,7 +1849,7 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -1820,11 +1957,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -1835,11 +1967,6 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
@@ -1871,9 +1998,6 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2272,23 +2396,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>11430</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>598713</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>11430</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>370114</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>4354</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BF8B72D-AB5A-5E10-0B84-0CCDBEF3D45F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82796868-E333-EEE0-B037-AA9AA566D28C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3024,7 +3148,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0519DB-39C6-4963-B577-A1DDE442233F}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.5546875" customWidth="1"/>
@@ -3065,17 +3189,17 @@
         <v>446196</v>
       </c>
       <c r="C2">
-        <v>115.9</v>
+        <v>118.85</v>
       </c>
       <c r="D2">
-        <v>115.21</v>
+        <v>118.42</v>
       </c>
       <c r="E2">
-        <v>114.63</v>
+        <v>118.06</v>
       </c>
       <c r="F2" s="1">
         <f>AVERAGE(C2:E2)</f>
-        <v>115.24666666666667</v>
+        <v>118.44333333333333</v>
       </c>
       <c r="H2" s="3">
         <v>20</v>
@@ -3089,17 +3213,17 @@
         <v>2557912</v>
       </c>
       <c r="C3">
-        <v>106.71</v>
+        <v>105.44</v>
       </c>
       <c r="D3">
-        <v>106.04</v>
+        <v>104.81</v>
       </c>
       <c r="E3">
-        <v>105.47</v>
+        <v>104.73</v>
       </c>
       <c r="F3" s="1">
         <f t="shared" ref="F3:F7" si="0">AVERAGE(C3:E3)</f>
-        <v>106.07333333333334</v>
+        <v>104.99333333333334</v>
       </c>
       <c r="H3" s="3">
         <v>20</v>
@@ -3113,17 +3237,17 @@
         <v>6588388</v>
       </c>
       <c r="C4">
-        <v>96.89</v>
+        <v>88.74</v>
       </c>
       <c r="D4">
-        <v>96.23</v>
+        <v>88.25</v>
       </c>
       <c r="E4">
-        <v>95.4</v>
+        <v>87.78</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" si="0"/>
-        <v>96.173333333333332</v>
+        <v>88.256666666666661</v>
       </c>
       <c r="H4" s="3">
         <v>20</v>
@@ -3137,17 +3261,17 @@
         <v>12503168</v>
       </c>
       <c r="C5">
-        <v>80.97</v>
+        <v>76.7</v>
       </c>
       <c r="D5">
-        <v>81.260000000000005</v>
+        <v>76.66</v>
       </c>
       <c r="E5">
-        <v>80.55</v>
+        <v>76.41</v>
       </c>
       <c r="F5" s="1">
         <f t="shared" si="0"/>
-        <v>80.926666666666677</v>
+        <v>76.59</v>
       </c>
       <c r="H5" s="3">
         <v>20</v>
@@ -3161,17 +3285,17 @@
         <v>20099300</v>
       </c>
       <c r="C6">
-        <v>67.88</v>
+        <v>71.540000000000006</v>
       </c>
       <c r="D6">
-        <v>68.77</v>
+        <v>71.05</v>
       </c>
       <c r="E6">
-        <v>67.41</v>
+        <v>70.900000000000006</v>
       </c>
       <c r="F6" s="1">
         <f t="shared" si="0"/>
-        <v>68.02</v>
+        <v>71.163333333333341</v>
       </c>
       <c r="H6" s="3">
         <v>20</v>
@@ -3185,44 +3309,181 @@
         <v>29901464</v>
       </c>
       <c r="C7">
-        <v>58.03</v>
+        <v>65.95</v>
       </c>
       <c r="D7">
-        <v>56.73</v>
+        <v>65.22</v>
       </c>
       <c r="E7">
-        <v>56.16</v>
+        <v>64.05</v>
       </c>
       <c r="F7" s="1">
         <f t="shared" si="0"/>
-        <v>56.973333333333329</v>
+        <v>65.073333333333338</v>
       </c>
       <c r="H7" s="3">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="4">
-        <v>40374324</v>
-      </c>
-      <c r="C8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="B8" s="4"/>
+      <c r="F8" s="1"/>
       <c r="H8" s="3">
         <v>20</v>
       </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="4">
+        <v>446196</v>
+      </c>
+      <c r="C11">
+        <v>120.42</v>
+      </c>
+      <c r="D11">
+        <v>119.66</v>
+      </c>
+      <c r="E11">
+        <v>118.99</v>
+      </c>
+      <c r="F11" s="1">
+        <f>AVERAGE(C11:E11)</f>
+        <v>119.69</v>
+      </c>
+      <c r="H11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="4">
+        <v>2557912</v>
+      </c>
+      <c r="C12">
+        <v>109.89</v>
+      </c>
+      <c r="D12">
+        <v>109.21</v>
+      </c>
+      <c r="E12">
+        <v>108.85</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" ref="F12:F16" si="1">AVERAGE(C12:E12)</f>
+        <v>109.31666666666666</v>
+      </c>
+      <c r="H12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="4">
+        <v>6588388</v>
+      </c>
+      <c r="C13">
+        <v>91.78</v>
+      </c>
+      <c r="D13">
+        <v>91.47</v>
+      </c>
+      <c r="E13">
+        <v>91.09</v>
+      </c>
+      <c r="F13" s="1">
+        <f t="shared" si="1"/>
+        <v>91.446666666666673</v>
+      </c>
+      <c r="H13" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="4">
+        <v>12503168</v>
+      </c>
+      <c r="C14">
+        <v>80.02</v>
+      </c>
+      <c r="D14">
+        <v>79.72</v>
+      </c>
+      <c r="E14">
+        <v>79.459999999999994</v>
+      </c>
+      <c r="F14" s="1">
+        <f t="shared" si="1"/>
+        <v>79.733333333333334</v>
+      </c>
+      <c r="H14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="4">
+        <v>20099300</v>
+      </c>
+      <c r="C15">
+        <v>73.09</v>
+      </c>
+      <c r="D15">
+        <v>73.12</v>
+      </c>
+      <c r="E15">
+        <v>72.959999999999994</v>
+      </c>
+      <c r="F15" s="1">
+        <f t="shared" si="1"/>
+        <v>73.056666666666672</v>
+      </c>
+      <c r="H15" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>29901464</v>
+      </c>
+      <c r="C16">
+        <v>65.760000000000005</v>
+      </c>
+      <c r="D16">
+        <v>65.849999999999994</v>
+      </c>
+      <c r="E16">
+        <v>66.239999999999995</v>
+      </c>
+      <c r="F16" s="1">
+        <f t="shared" si="1"/>
+        <v>65.95</v>
+      </c>
+      <c r="H16" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="4"/>
+      <c r="F17" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>